<commit_message>
align tutorial code with workbook results
</commit_message>
<xml_diff>
--- a/site/assets/examples/05-edit-a-template.xlsx
+++ b/site/assets/examples/05-edit-a-template.xlsx
@@ -136,14 +136,14 @@
     <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>INVOICE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Fill the highlighted cells and keep the original design.</t>

</xml_diff>